<commit_message>
db prep scripts for cutover
</commit_message>
<xml_diff>
--- a/uploads/Clients_1776399772.xlsx
+++ b/uploads/Clients_1776399772.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD17074-BD95-42E2-A068-276B8441594A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F4B2DA-0023-4F9A-8D4B-467D1B284E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clients" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="300">
   <si>
     <t>Name</t>
   </si>
@@ -843,6 +843,78 @@
   </si>
   <si>
     <t>BJC PCL</t>
+  </si>
+  <si>
+    <t>TCP</t>
+  </si>
+  <si>
+    <t>DFI</t>
+  </si>
+  <si>
+    <t>Matahari</t>
+  </si>
+  <si>
+    <t>Indonesia</t>
+  </si>
+  <si>
+    <t>Seven.sa</t>
+  </si>
+  <si>
+    <t>Heritage Grocer Group</t>
+  </si>
+  <si>
+    <t>Alix Partners</t>
+  </si>
+  <si>
+    <t>IMT</t>
+  </si>
+  <si>
+    <t>Transportation</t>
+  </si>
+  <si>
+    <t>TCC Group</t>
+  </si>
+  <si>
+    <t>The Mall Group</t>
+  </si>
+  <si>
+    <t>Paneco</t>
+  </si>
+  <si>
+    <t>Olivia</t>
+  </si>
+  <si>
+    <t>Right Roofing</t>
+  </si>
+  <si>
+    <t>Startup</t>
+  </si>
+  <si>
+    <t>Maison</t>
+  </si>
+  <si>
+    <t>Conglomerate</t>
+  </si>
+  <si>
+    <t>AIS</t>
+  </si>
+  <si>
+    <t>Telecom</t>
+  </si>
+  <si>
+    <t>Bath &amp; Body Works</t>
+  </si>
+  <si>
+    <t>Dubai</t>
+  </si>
+  <si>
+    <t>United Arab Emirates</t>
+  </si>
+  <si>
+    <t>Ahold Int'l</t>
+  </si>
+  <si>
+    <t>Bank Vista</t>
   </si>
 </sst>
 </file>
@@ -1270,7 +1342,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F226"/>
+  <dimension ref="A1:F244"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1437,7 +1509,7 @@
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1610,7 +1682,7 @@
         <v>8</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1652,7 +1724,7 @@
         <v>8</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1765,7 +1837,9 @@
       <c r="C34" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F34" s="3"/>
+      <c r="F34" s="3" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="35" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
@@ -1778,7 +1852,7 @@
         <v>50</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1792,7 +1866,7 @@
         <v>50</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1806,7 +1880,7 @@
         <v>50</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1820,7 +1894,7 @@
         <v>50</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1934,7 +2008,7 @@
         <v>13</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1977,7 +2051,7 @@
         <v>13</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2005,7 +2079,7 @@
         <v>78</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2061,7 +2135,7 @@
         <v>8</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2132,7 +2206,7 @@
         <v>88</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2146,7 +2220,7 @@
         <v>13</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2160,7 +2234,7 @@
         <v>8</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2230,7 +2304,7 @@
         <v>50</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2244,7 +2318,7 @@
         <v>7</v>
       </c>
       <c r="F68" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2530,7 +2604,7 @@
         <v>50</v>
       </c>
       <c r="F88" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2716,7 +2790,7 @@
         <v>8</v>
       </c>
       <c r="F101" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2744,7 +2818,7 @@
         <v>50</v>
       </c>
       <c r="F103" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="104" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2774,7 +2848,7 @@
         <v>73</v>
       </c>
       <c r="F105" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2803,7 +2877,7 @@
         <v>50</v>
       </c>
       <c r="F107" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="108" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2818,7 +2892,7 @@
       </c>
       <c r="D108" s="3"/>
       <c r="F108" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="109" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2904,7 +2978,7 @@
       </c>
       <c r="E114" s="3"/>
       <c r="F114" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="115" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2974,6 +3048,9 @@
         <v>19</v>
       </c>
       <c r="E119" s="3"/>
+      <c r="F119" s="7" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="120" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
@@ -3029,7 +3106,7 @@
         <v>50</v>
       </c>
       <c r="F123" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="124" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3186,7 +3263,7 @@
         <v>8</v>
       </c>
       <c r="F134" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="135" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3258,7 +3335,7 @@
       </c>
       <c r="E139" s="3"/>
       <c r="F139" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="140" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3370,7 +3447,7 @@
         <v>8</v>
       </c>
       <c r="F147" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="148" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3470,7 +3547,7 @@
         <v>38</v>
       </c>
       <c r="F154" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
@@ -3484,7 +3561,7 @@
         <v>38</v>
       </c>
       <c r="F155" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
@@ -3512,7 +3589,7 @@
         <v>19</v>
       </c>
       <c r="F157" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
@@ -3526,7 +3603,7 @@
         <v>13</v>
       </c>
       <c r="F158" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.3">
@@ -3811,7 +3888,7 @@
         <v>19</v>
       </c>
       <c r="F178" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
@@ -3825,7 +3902,7 @@
         <v>19</v>
       </c>
       <c r="F179" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
@@ -3869,7 +3946,7 @@
         <v>240</v>
       </c>
       <c r="F182" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
@@ -3883,7 +3960,7 @@
         <v>50</v>
       </c>
       <c r="F183" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
@@ -4150,7 +4227,7 @@
         <v>50</v>
       </c>
       <c r="F202" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.3">
@@ -4347,7 +4424,7 @@
         <v>19</v>
       </c>
       <c r="F216" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.3">
@@ -4375,7 +4452,7 @@
         <v>19</v>
       </c>
       <c r="F218" s="3" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.3">
@@ -4490,6 +4567,243 @@
       </c>
       <c r="E226" s="3"/>
       <c r="F226" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A227" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B227" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F227" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A228" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B228" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C228" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F228" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A229" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B229" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C229" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F229" s="7" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A230" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B230" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F230" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A231" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B231" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C231" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F231" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="232" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A232" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B232" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C232" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F232" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A233" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B233" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C233" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="F233" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="234" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A234" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B234" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F234" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="235" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A235" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B235" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F235" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="236" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A236" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B236" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F236" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="237" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A237" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B237" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C237" t="s">
+        <v>290</v>
+      </c>
+      <c r="F237" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="238" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A238" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B238" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C238" t="s">
+        <v>105</v>
+      </c>
+      <c r="F238" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="239" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A239" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B239" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C239" t="s">
+        <v>292</v>
+      </c>
+      <c r="F239" s="7" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="240" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A240" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B240" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C240" t="s">
+        <v>294</v>
+      </c>
+      <c r="F240" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="241" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A241" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B241" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C241" t="s">
+        <v>19</v>
+      </c>
+      <c r="F241" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="242" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A242" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B242" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F242" s="7" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="243" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A243" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="B243" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C243" t="s">
+        <v>19</v>
+      </c>
+      <c r="F243" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="244" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A244" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B244" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C244" t="s">
+        <v>140</v>
+      </c>
+      <c r="F244" s="7" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>